<commit_message>
Adapt MAGNET_CarbonLeak regional aggregation
</commit_message>
<xml_diff>
--- a/linking_pipeline/data/input/m_Country.xlsx
+++ b/linking_pipeline/data/input/m_Country.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\honkomp\PycharmProjects\gfpmpt_linking_pipeline\linking_pipeline\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201AAF8B-0188-4F5F-8C35-0D85F01C4392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35686155-2688-4CE4-8410-C3A12DB552FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="4392" windowWidth="21960" windowHeight="11880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m_Country" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">m_Country!$A$1:$AG$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">m_Country!$A$1:$AH$1</definedName>
     <definedName name="m_Country">m_Country!$A$1:$AG$193</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4619" uniqueCount="1024">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4619" uniqueCount="1023">
   <si>
     <t>ID</t>
   </si>
@@ -3097,9 +3097,6 @@
   </si>
   <si>
     <t>ROW_NWTO</t>
-  </si>
-  <si>
-    <t>Asia</t>
   </si>
   <si>
     <t>CSAM</t>
@@ -3588,7 +3585,7 @@
         <v>1002</v>
       </c>
       <c r="H1" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="I1" t="s">
         <v>5</v>
@@ -3660,7 +3657,7 @@
         <v>27</v>
       </c>
       <c r="AF1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="AG1" t="s">
         <v>28</v>
@@ -3847,7 +3844,7 @@
         <v>34</v>
       </c>
       <c r="AH3" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -3945,7 +3942,7 @@
         <v>50</v>
       </c>
       <c r="AH4" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -4046,7 +4043,7 @@
         <v>57</v>
       </c>
       <c r="AH5" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -4144,7 +4141,7 @@
         <v>63</v>
       </c>
       <c r="AH6" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -4242,7 +4239,7 @@
         <v>70</v>
       </c>
       <c r="AH7" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -4340,7 +4337,7 @@
         <v>75</v>
       </c>
       <c r="AH8" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -4441,7 +4438,7 @@
         <v>80</v>
       </c>
       <c r="AH9" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -4539,7 +4536,7 @@
         <v>86</v>
       </c>
       <c r="AH10" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -4637,7 +4634,7 @@
         <v>91</v>
       </c>
       <c r="AH11" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -4735,7 +4732,7 @@
         <v>96</v>
       </c>
       <c r="AH12" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -4836,7 +4833,7 @@
         <v>105</v>
       </c>
       <c r="AH13" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -4937,7 +4934,7 @@
         <v>106</v>
       </c>
       <c r="AH14" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -5035,7 +5032,7 @@
         <v>111</v>
       </c>
       <c r="AH15" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -5133,7 +5130,7 @@
         <v>115</v>
       </c>
       <c r="AH16" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -5231,7 +5228,7 @@
         <v>120</v>
       </c>
       <c r="AH17" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -5332,7 +5329,7 @@
         <v>125</v>
       </c>
       <c r="AH18" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -5433,7 +5430,7 @@
         <v>131</v>
       </c>
       <c r="AH19" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -5531,7 +5528,7 @@
         <v>135</v>
       </c>
       <c r="AH20" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -5632,7 +5629,7 @@
         <v>139</v>
       </c>
       <c r="AH21" t="s">
-        <v>141</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -5730,7 +5727,7 @@
         <v>144</v>
       </c>
       <c r="AH22" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -5828,7 +5825,7 @@
         <v>149</v>
       </c>
       <c r="AH23" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -5929,7 +5926,7 @@
         <v>153</v>
       </c>
       <c r="AH24" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -6027,7 +6024,7 @@
         <v>158</v>
       </c>
       <c r="AH25" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -6125,7 +6122,7 @@
         <v>164</v>
       </c>
       <c r="AH26" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -6223,7 +6220,7 @@
         <v>172</v>
       </c>
       <c r="AH27" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -6321,7 +6318,7 @@
         <v>173</v>
       </c>
       <c r="AH28" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -6422,7 +6419,7 @@
         <v>178</v>
       </c>
       <c r="AH29" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -6520,7 +6517,7 @@
         <v>183</v>
       </c>
       <c r="AH30" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -6618,7 +6615,7 @@
         <v>187</v>
       </c>
       <c r="AH31" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -6716,7 +6713,7 @@
         <v>191</v>
       </c>
       <c r="AH32" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -6817,7 +6814,7 @@
         <v>196</v>
       </c>
       <c r="AH33" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -6915,7 +6912,7 @@
         <v>201</v>
       </c>
       <c r="AH34" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -7013,7 +7010,7 @@
         <v>206</v>
       </c>
       <c r="AH35" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -7114,7 +7111,7 @@
         <v>210</v>
       </c>
       <c r="AH36" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -7209,7 +7206,7 @@
         <v>215</v>
       </c>
       <c r="AH37" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -7307,7 +7304,7 @@
         <v>220</v>
       </c>
       <c r="AH38" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -7405,7 +7402,7 @@
         <v>225</v>
       </c>
       <c r="AH39" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -7503,7 +7500,7 @@
         <v>229</v>
       </c>
       <c r="AH40" t="s">
-        <v>231</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -7601,7 +7598,7 @@
         <v>234</v>
       </c>
       <c r="AH41" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -7699,7 +7696,7 @@
         <v>238</v>
       </c>
       <c r="AH42" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -7797,7 +7794,7 @@
         <v>242</v>
       </c>
       <c r="AH43" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -7895,7 +7892,7 @@
         <v>247</v>
       </c>
       <c r="AH44" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -7993,7 +7990,7 @@
         <v>251</v>
       </c>
       <c r="AH45" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -8091,7 +8088,7 @@
         <v>260</v>
       </c>
       <c r="AH46" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -8192,7 +8189,7 @@
         <v>261</v>
       </c>
       <c r="AH47" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -8290,7 +8287,7 @@
         <v>266</v>
       </c>
       <c r="AH48" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -8391,7 +8388,7 @@
         <v>271</v>
       </c>
       <c r="AH49" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -8489,7 +8486,7 @@
         <v>280</v>
       </c>
       <c r="AH50" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -8590,7 +8587,7 @@
         <v>281</v>
       </c>
       <c r="AH51" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -8691,7 +8688,7 @@
         <v>286</v>
       </c>
       <c r="AH52" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -8869,7 +8866,7 @@
         <v>294</v>
       </c>
       <c r="AH54" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -8967,7 +8964,7 @@
         <v>302</v>
       </c>
       <c r="AH55" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -9065,7 +9062,7 @@
         <v>306</v>
       </c>
       <c r="AH56" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -9261,7 +9258,7 @@
         <v>317</v>
       </c>
       <c r="AH58" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -9362,7 +9359,7 @@
         <v>321</v>
       </c>
       <c r="AH59" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -9460,7 +9457,7 @@
         <v>326</v>
       </c>
       <c r="AH60" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -9558,7 +9555,7 @@
         <v>330</v>
       </c>
       <c r="AH61" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -9656,7 +9653,7 @@
         <v>334</v>
       </c>
       <c r="AH62" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -9757,7 +9754,7 @@
         <v>339</v>
       </c>
       <c r="AH63" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -9858,7 +9855,7 @@
         <v>344</v>
       </c>
       <c r="AH64" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -9956,7 +9953,7 @@
         <v>349</v>
       </c>
       <c r="AH65" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -10057,7 +10054,7 @@
         <v>353</v>
       </c>
       <c r="AH66" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -10155,7 +10152,7 @@
         <v>358</v>
       </c>
       <c r="AH67" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -10250,7 +10247,7 @@
         <v>363</v>
       </c>
       <c r="AH68" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -10351,7 +10348,7 @@
         <v>367</v>
       </c>
       <c r="AH69" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -10443,7 +10440,7 @@
         <v>372</v>
       </c>
       <c r="AH70" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -10541,7 +10538,7 @@
         <v>375</v>
       </c>
       <c r="AH71" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -10642,7 +10639,7 @@
         <v>380</v>
       </c>
       <c r="AH72" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -10740,7 +10737,7 @@
         <v>389</v>
       </c>
       <c r="AH73" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -10838,7 +10835,7 @@
         <v>390</v>
       </c>
       <c r="AH74" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -11117,7 +11114,7 @@
         <v>404</v>
       </c>
       <c r="AH77" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -11215,7 +11212,7 @@
         <v>409</v>
       </c>
       <c r="AH78" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -11518,7 +11515,7 @@
         <v>426</v>
       </c>
       <c r="AH81" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -11619,7 +11616,7 @@
         <v>431</v>
       </c>
       <c r="AH82" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -11913,7 +11910,7 @@
         <v>445</v>
       </c>
       <c r="AH85" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -12014,7 +12011,7 @@
         <v>450</v>
       </c>
       <c r="AH86" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -12213,7 +12210,7 @@
         <v>459</v>
       </c>
       <c r="AH88" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -12311,7 +12308,7 @@
         <v>469</v>
       </c>
       <c r="AH89" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -12489,7 +12486,7 @@
         <v>473</v>
       </c>
       <c r="AH91" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -12587,7 +12584,7 @@
         <v>481</v>
       </c>
       <c r="AH92" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -12688,7 +12685,7 @@
         <v>487</v>
       </c>
       <c r="AH93" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -12786,7 +12783,7 @@
         <v>492</v>
       </c>
       <c r="AH94" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -12884,7 +12881,7 @@
         <v>496</v>
       </c>
       <c r="AH95" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -12982,7 +12979,7 @@
         <v>502</v>
       </c>
       <c r="AH96" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -13178,7 +13175,7 @@
         <v>512</v>
       </c>
       <c r="AH98" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -13276,7 +13273,7 @@
         <v>518</v>
       </c>
       <c r="AH99" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -13772,7 +13769,7 @@
         <v>542</v>
       </c>
       <c r="AH104" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -13968,7 +13965,7 @@
         <v>553</v>
       </c>
       <c r="AH106" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -14066,7 +14063,7 @@
         <v>564</v>
       </c>
       <c r="AH107" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -14164,7 +14161,7 @@
         <v>570</v>
       </c>
       <c r="AH108" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -14262,7 +14259,7 @@
         <v>571</v>
       </c>
       <c r="AH109" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -14363,7 +14360,7 @@
         <v>581</v>
       </c>
       <c r="AH110" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -14559,7 +14556,7 @@
         <v>586</v>
       </c>
       <c r="AH112" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -14660,7 +14657,7 @@
         <v>591</v>
       </c>
       <c r="AH113" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -14758,7 +14755,7 @@
         <v>597</v>
       </c>
       <c r="AH114" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -14859,7 +14856,7 @@
         <v>602</v>
       </c>
       <c r="AH115" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -14957,7 +14954,7 @@
         <v>606</v>
       </c>
       <c r="AH116" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -15055,7 +15052,7 @@
         <v>611</v>
       </c>
       <c r="AH117" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -15153,7 +15150,7 @@
         <v>616</v>
       </c>
       <c r="AH118" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -15254,7 +15251,7 @@
         <v>621</v>
       </c>
       <c r="AH119" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -15352,7 +15349,7 @@
         <v>626</v>
       </c>
       <c r="AH120" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -15450,7 +15447,7 @@
         <v>631</v>
       </c>
       <c r="AH121" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -15548,7 +15545,7 @@
         <v>636</v>
       </c>
       <c r="AH122" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -15649,7 +15646,7 @@
         <v>641</v>
       </c>
       <c r="AH123" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -15845,7 +15842,7 @@
         <v>650</v>
       </c>
       <c r="AH125" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -16041,7 +16038,7 @@
         <v>660</v>
       </c>
       <c r="AH127" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -16142,7 +16139,7 @@
         <v>665</v>
       </c>
       <c r="AH128" t="s">
-        <v>1013</v>
+        <v>470</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -17582,7 +17579,7 @@
         <v>730</v>
       </c>
       <c r="AH143" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -17680,7 +17677,7 @@
         <v>738</v>
       </c>
       <c r="AH144" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -17778,7 +17775,7 @@
         <v>744</v>
       </c>
       <c r="AH145" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -18072,7 +18069,7 @@
         <v>760</v>
       </c>
       <c r="AH148" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -18170,7 +18167,7 @@
         <v>765</v>
       </c>
       <c r="AH149" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -18268,7 +18265,7 @@
         <v>770</v>
       </c>
       <c r="AH150" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -18366,7 +18363,7 @@
         <v>776</v>
       </c>
       <c r="AH151" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -18464,7 +18461,7 @@
         <v>781</v>
       </c>
       <c r="AH152" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -18660,7 +18657,7 @@
         <v>790</v>
       </c>
       <c r="AH154" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -18856,7 +18853,7 @@
         <v>800</v>
       </c>
       <c r="AH156" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -18954,7 +18951,7 @@
         <v>805</v>
       </c>
       <c r="AH157" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -19052,7 +19049,7 @@
         <v>810</v>
       </c>
       <c r="AH158" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -19444,7 +19441,7 @@
         <v>829</v>
       </c>
       <c r="AH162" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -19640,7 +19637,7 @@
         <v>840</v>
       </c>
       <c r="AH164" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -19934,7 +19931,7 @@
         <v>855</v>
       </c>
       <c r="AH167" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -20032,7 +20029,7 @@
         <v>860</v>
       </c>
       <c r="AH168" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -20130,7 +20127,7 @@
         <v>865</v>
       </c>
       <c r="AH169" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -20228,7 +20225,7 @@
         <v>870</v>
       </c>
       <c r="AH170" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -20602,7 +20599,7 @@
         <v>888</v>
       </c>
       <c r="AH174" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -20896,7 +20893,7 @@
         <v>908</v>
       </c>
       <c r="AH177" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -20994,7 +20991,7 @@
         <v>914</v>
       </c>
       <c r="AH178" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -21190,7 +21187,7 @@
         <v>924</v>
       </c>
       <c r="AH180" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -21288,7 +21285,7 @@
         <v>929</v>
       </c>
       <c r="AH181" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -21386,7 +21383,7 @@
         <v>934</v>
       </c>
       <c r="AH182" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -21680,7 +21677,7 @@
         <v>950</v>
       </c>
       <c r="AH185" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -21778,7 +21775,7 @@
         <v>955</v>
       </c>
       <c r="AH186" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -21974,7 +21971,7 @@
         <v>964</v>
       </c>
       <c r="AH188" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -22297,7 +22294,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG194" xr:uid="{FC0DF5AA-9463-4F44-A221-46D8695B8D1F}"/>
+  <autoFilter ref="A1:AH1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update MAGNET country aggregation for CarbonLeak project
</commit_message>
<xml_diff>
--- a/linking_pipeline/data/input/m_Country.xlsx
+++ b/linking_pipeline/data/input/m_Country.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\honkomp\PycharmProjects\gfpmpt_linking_pipeline\linking_pipeline\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\honkomp\PycharmProjects\GitHub\CGE_linking_pipeline\linking_pipeline\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B235FDE8-161F-42DE-B80B-4500A56967CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D78D6A0-3149-4E6D-A6A1-D2B546D38120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2775" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="345" yWindow="555" windowWidth="23040" windowHeight="12270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m_Country" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">m_Country!$A$1:$AI$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">m_Country!$A$1:$AI$193</definedName>
     <definedName name="m_Country">m_Country!$A$1:$AH$193</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -3108,9 +3108,6 @@
     <t>ROW_WTO</t>
   </si>
   <si>
-    <t>EU20</t>
-  </si>
-  <si>
     <t>EFTA</t>
   </si>
   <si>
@@ -3130,6 +3127,9 @@
   </si>
   <si>
     <t>DART-BIO_BioSDG_cp</t>
+  </si>
+  <si>
+    <t>EU27</t>
   </si>
 </sst>
 </file>
@@ -3536,36 +3536,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI193"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="9" width="22.44140625" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" customWidth="1"/>
-    <col min="12" max="12" width="18.44140625" customWidth="1"/>
-    <col min="13" max="13" width="22.6640625" customWidth="1"/>
-    <col min="14" max="14" width="23.6640625" customWidth="1"/>
-    <col min="15" max="15" width="13" customWidth="1"/>
-    <col min="16" max="16" width="9.5546875" customWidth="1"/>
-    <col min="17" max="17" width="21" customWidth="1"/>
-    <col min="18" max="18" width="11.88671875" customWidth="1"/>
-    <col min="19" max="19" width="9.44140625" customWidth="1"/>
-    <col min="20" max="20" width="11.88671875" customWidth="1"/>
-    <col min="21" max="21" width="9.109375" customWidth="1"/>
-    <col min="22" max="22" width="9.6640625" customWidth="1"/>
-    <col min="23" max="27" width="9.109375" customWidth="1"/>
-    <col min="28" max="28" width="11.5546875" customWidth="1"/>
-    <col min="29" max="29" width="20.33203125" customWidth="1"/>
-    <col min="30" max="31" width="9.109375" customWidth="1"/>
-    <col min="32" max="32" width="24.33203125" customWidth="1"/>
-    <col min="33" max="33" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="39.44140625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" hidden="1" customWidth="1"/>
+    <col min="5" max="9" width="22.42578125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="13" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="9.5703125" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="21" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="9.42578125" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="11.85546875" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="9.7109375" hidden="1" customWidth="1"/>
+    <col min="23" max="27" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="11.5703125" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="20.28515625" hidden="1" customWidth="1"/>
+    <col min="30" max="31" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="24.28515625" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="39.42578125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3588,10 +3588,10 @@
         <v>1002</v>
       </c>
       <c r="H1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="I1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="J1" t="s">
         <v>5</v>
@@ -3663,7 +3663,7 @@
         <v>27</v>
       </c>
       <c r="AG1" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="AH1" t="s">
         <v>28</v>
@@ -3672,7 +3672,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3758,7 +3758,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3856,10 +3856,10 @@
         <v>34</v>
       </c>
       <c r="AI3" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3957,10 +3957,10 @@
         <v>50</v>
       </c>
       <c r="AI4" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4061,10 +4061,10 @@
         <v>57</v>
       </c>
       <c r="AI5" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4162,10 +4162,10 @@
         <v>63</v>
       </c>
       <c r="AI6" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4263,10 +4263,10 @@
         <v>70</v>
       </c>
       <c r="AI7" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -4364,10 +4364,10 @@
         <v>75</v>
       </c>
       <c r="AI8" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4468,10 +4468,10 @@
         <v>80</v>
       </c>
       <c r="AI9" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4569,10 +4569,10 @@
         <v>86</v>
       </c>
       <c r="AI10" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4670,10 +4670,10 @@
         <v>91</v>
       </c>
       <c r="AI11" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4771,10 +4771,10 @@
         <v>96</v>
       </c>
       <c r="AI12" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4875,10 +4875,10 @@
         <v>105</v>
       </c>
       <c r="AI13" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4979,10 +4979,10 @@
         <v>106</v>
       </c>
       <c r="AI14" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -5080,10 +5080,10 @@
         <v>111</v>
       </c>
       <c r="AI15" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -5181,10 +5181,10 @@
         <v>115</v>
       </c>
       <c r="AI16" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -5282,10 +5282,10 @@
         <v>120</v>
       </c>
       <c r="AI17" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -5386,10 +5386,10 @@
         <v>125</v>
       </c>
       <c r="AI18" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -5490,10 +5490,10 @@
         <v>131</v>
       </c>
       <c r="AI19" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -5591,10 +5591,10 @@
         <v>135</v>
       </c>
       <c r="AI20" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -5695,10 +5695,10 @@
         <v>139</v>
       </c>
       <c r="AI21" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -5796,10 +5796,10 @@
         <v>144</v>
       </c>
       <c r="AI22" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -5897,10 +5897,10 @@
         <v>149</v>
       </c>
       <c r="AI23" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -6001,10 +6001,10 @@
         <v>153</v>
       </c>
       <c r="AI24" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -6102,10 +6102,10 @@
         <v>158</v>
       </c>
       <c r="AI25" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -6203,10 +6203,10 @@
         <v>164</v>
       </c>
       <c r="AI26" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -6304,10 +6304,10 @@
         <v>172</v>
       </c>
       <c r="AI27" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -6405,10 +6405,10 @@
         <v>173</v>
       </c>
       <c r="AI28" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -6509,10 +6509,10 @@
         <v>178</v>
       </c>
       <c r="AI29" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -6610,10 +6610,10 @@
         <v>183</v>
       </c>
       <c r="AI30" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -6711,10 +6711,10 @@
         <v>187</v>
       </c>
       <c r="AI31" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -6812,10 +6812,10 @@
         <v>191</v>
       </c>
       <c r="AI32" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -6916,10 +6916,10 @@
         <v>196</v>
       </c>
       <c r="AI33" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -7017,10 +7017,10 @@
         <v>201</v>
       </c>
       <c r="AI34" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -7118,10 +7118,10 @@
         <v>206</v>
       </c>
       <c r="AI35" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -7222,10 +7222,10 @@
         <v>210</v>
       </c>
       <c r="AI36" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -7320,10 +7320,10 @@
         <v>215</v>
       </c>
       <c r="AI37" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -7421,10 +7421,10 @@
         <v>220</v>
       </c>
       <c r="AI38" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -7522,10 +7522,10 @@
         <v>225</v>
       </c>
       <c r="AI39" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -7623,10 +7623,10 @@
         <v>229</v>
       </c>
       <c r="AI40" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -7724,10 +7724,10 @@
         <v>234</v>
       </c>
       <c r="AI41" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -7825,10 +7825,10 @@
         <v>238</v>
       </c>
       <c r="AI42" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -7926,10 +7926,10 @@
         <v>242</v>
       </c>
       <c r="AI43" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -8027,10 +8027,10 @@
         <v>247</v>
       </c>
       <c r="AI44" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -8128,10 +8128,10 @@
         <v>251</v>
       </c>
       <c r="AI45" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -8229,10 +8229,10 @@
         <v>260</v>
       </c>
       <c r="AI46" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -8333,10 +8333,10 @@
         <v>261</v>
       </c>
       <c r="AI47" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -8434,10 +8434,10 @@
         <v>266</v>
       </c>
       <c r="AI48" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -8538,10 +8538,10 @@
         <v>271</v>
       </c>
       <c r="AI49" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -8639,10 +8639,10 @@
         <v>280</v>
       </c>
       <c r="AI50" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -8743,10 +8743,10 @@
         <v>281</v>
       </c>
       <c r="AI51" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -8847,10 +8847,10 @@
         <v>286</v>
       </c>
       <c r="AI52" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -8933,7 +8933,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -9034,7 +9034,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -9135,7 +9135,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -9236,7 +9236,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -9337,7 +9337,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -9438,7 +9438,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -9542,7 +9542,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -9643,7 +9643,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -9744,7 +9744,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="62" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -9845,7 +9845,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -9949,7 +9949,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -10053,7 +10053,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="65" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -10154,7 +10154,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -10359,7 +10359,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -10454,10 +10454,10 @@
         <v>363</v>
       </c>
       <c r="AI68" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -10561,7 +10561,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -10656,7 +10656,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -10757,7 +10757,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -10861,7 +10861,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -10962,7 +10962,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -11063,7 +11063,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="75" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -11164,7 +11164,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="76" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -11247,7 +11247,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="77" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -11351,7 +11351,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="78" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -11452,7 +11452,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="79" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -11556,7 +11556,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="80" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -11660,7 +11660,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="81" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -11764,7 +11764,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="82" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -11868,7 +11868,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="83" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -11966,7 +11966,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="84" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -12067,7 +12067,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="85" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -12171,7 +12171,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="86" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -12275,7 +12275,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="87" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -12379,7 +12379,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="88" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -12480,7 +12480,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="89" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -12581,7 +12581,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="90" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -12664,7 +12664,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="91" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -12765,7 +12765,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="92" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -12863,10 +12863,10 @@
         <v>481</v>
       </c>
       <c r="AI92" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="93" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -12970,7 +12970,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="94" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -13071,7 +13071,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="95" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -13172,7 +13172,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="96" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -13273,7 +13273,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="97" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -13374,7 +13374,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="98" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -13472,10 +13472,10 @@
         <v>512</v>
       </c>
       <c r="AI98" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="99" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -13576,7 +13576,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="100" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -13680,7 +13680,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="101" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -13784,7 +13784,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="102" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -13885,7 +13885,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="103" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -13986,7 +13986,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="104" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -14084,10 +14084,10 @@
         <v>542</v>
       </c>
       <c r="AI104" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="105" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -14188,7 +14188,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="106" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -14286,10 +14286,10 @@
         <v>553</v>
       </c>
       <c r="AI106" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="107" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -14390,7 +14390,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="108" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -14491,7 +14491,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="109" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -14589,10 +14589,10 @@
         <v>571</v>
       </c>
       <c r="AI109" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="110" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -14696,7 +14696,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="111" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -14797,7 +14797,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="112" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -14898,7 +14898,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="113" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -15002,7 +15002,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="114" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -15103,7 +15103,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="115" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -15207,7 +15207,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="116" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -15308,7 +15308,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="117" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -15406,10 +15406,10 @@
         <v>611</v>
       </c>
       <c r="AI117" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="118" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -15510,7 +15510,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="119" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -15614,7 +15614,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="120" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -15712,10 +15712,10 @@
         <v>626</v>
       </c>
       <c r="AI120" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="121" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -15813,10 +15813,10 @@
         <v>631</v>
       </c>
       <c r="AI121" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="122" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -15917,7 +15917,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="123" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -16021,7 +16021,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="124" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -16122,7 +16122,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="125" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -16223,7 +16223,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="126" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -16324,7 +16324,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="127" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -16422,10 +16422,10 @@
         <v>660</v>
       </c>
       <c r="AI127" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
-    <row r="128" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -16529,7 +16529,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="129" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -16630,7 +16630,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="130" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -16713,7 +16713,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="131" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -16814,7 +16814,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="132" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -16912,7 +16912,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="133" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -17016,7 +17016,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="134" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
@@ -17117,7 +17117,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="135" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -17218,7 +17218,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="136" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
@@ -17319,7 +17319,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="137" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -17423,7 +17423,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="138" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -17524,7 +17524,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="139" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>138</v>
       </c>
@@ -17628,7 +17628,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="140" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
@@ -17729,7 +17729,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="141" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
@@ -17830,7 +17830,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="142" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
@@ -17913,7 +17913,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="143" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
@@ -18014,7 +18014,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="144" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
@@ -18112,10 +18112,10 @@
         <v>738</v>
       </c>
       <c r="AI144" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="145" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>144</v>
       </c>
@@ -18213,10 +18213,10 @@
         <v>744</v>
       </c>
       <c r="AI145" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="146" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>145</v>
       </c>
@@ -18317,7 +18317,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="147" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>146</v>
       </c>
@@ -18415,10 +18415,10 @@
         <v>754</v>
       </c>
       <c r="AI147" t="s">
-        <v>756</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="148" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>147</v>
       </c>
@@ -18516,10 +18516,10 @@
         <v>760</v>
       </c>
       <c r="AI148" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="149" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>148</v>
       </c>
@@ -18617,10 +18617,10 @@
         <v>765</v>
       </c>
       <c r="AI149" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="150" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>149</v>
       </c>
@@ -18718,10 +18718,10 @@
         <v>770</v>
       </c>
       <c r="AI150" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="151" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>150</v>
       </c>
@@ -18819,10 +18819,10 @@
         <v>776</v>
       </c>
       <c r="AI151" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="152" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>151</v>
       </c>
@@ -18920,10 +18920,10 @@
         <v>781</v>
       </c>
       <c r="AI152" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="153" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>152</v>
       </c>
@@ -19021,10 +19021,10 @@
         <v>785</v>
       </c>
       <c r="AI153" t="s">
-        <v>787</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="154" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>153</v>
       </c>
@@ -19122,10 +19122,10 @@
         <v>790</v>
       </c>
       <c r="AI154" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="155" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>154</v>
       </c>
@@ -19223,10 +19223,10 @@
         <v>795</v>
       </c>
       <c r="AI155" t="s">
-        <v>797</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="156" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>155</v>
       </c>
@@ -19324,10 +19324,10 @@
         <v>800</v>
       </c>
       <c r="AI156" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="157" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>156</v>
       </c>
@@ -19425,10 +19425,10 @@
         <v>805</v>
       </c>
       <c r="AI157" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="158" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>157</v>
       </c>
@@ -19526,10 +19526,10 @@
         <v>810</v>
       </c>
       <c r="AI158" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="159" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>158</v>
       </c>
@@ -19630,7 +19630,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="160" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>159</v>
       </c>
@@ -19731,7 +19731,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="161" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>160</v>
       </c>
@@ -19829,10 +19829,10 @@
         <v>824</v>
       </c>
       <c r="AI161" t="s">
-        <v>826</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="162" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>161</v>
       </c>
@@ -19930,10 +19930,10 @@
         <v>829</v>
       </c>
       <c r="AI162" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
-    <row r="163" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>162</v>
       </c>
@@ -20031,10 +20031,10 @@
         <v>835</v>
       </c>
       <c r="AI163" t="s">
-        <v>837</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="164" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>163</v>
       </c>
@@ -20132,10 +20132,10 @@
         <v>840</v>
       </c>
       <c r="AI164" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="165" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>164</v>
       </c>
@@ -20233,10 +20233,10 @@
         <v>845</v>
       </c>
       <c r="AI165" t="s">
-        <v>847</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="166" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>165</v>
       </c>
@@ -20334,10 +20334,10 @@
         <v>850</v>
       </c>
       <c r="AI166" t="s">
-        <v>852</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="167" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>166</v>
       </c>
@@ -20435,10 +20435,10 @@
         <v>855</v>
       </c>
       <c r="AI167" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="168" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>167</v>
       </c>
@@ -20536,10 +20536,10 @@
         <v>860</v>
       </c>
       <c r="AI168" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="169" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>168</v>
       </c>
@@ -20637,10 +20637,10 @@
         <v>865</v>
       </c>
       <c r="AI169" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="170" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>169</v>
       </c>
@@ -20738,10 +20738,10 @@
         <v>870</v>
       </c>
       <c r="AI170" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
-    <row r="171" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>170</v>
       </c>
@@ -20842,7 +20842,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="172" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>171</v>
       </c>
@@ -20943,7 +20943,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="173" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>172</v>
       </c>
@@ -21026,7 +21026,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="174" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>173</v>
       </c>
@@ -21127,7 +21127,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="175" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>174</v>
       </c>
@@ -21228,7 +21228,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="176" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>175</v>
       </c>
@@ -21329,7 +21329,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="177" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>176</v>
       </c>
@@ -21427,10 +21427,10 @@
         <v>908</v>
       </c>
       <c r="AI177" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="178" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>177</v>
       </c>
@@ -21531,7 +21531,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="179" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>178</v>
       </c>
@@ -21632,7 +21632,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="180" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>179</v>
       </c>
@@ -21733,7 +21733,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="181" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>180</v>
       </c>
@@ -21831,10 +21831,10 @@
         <v>929</v>
       </c>
       <c r="AI181" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="182" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>181</v>
       </c>
@@ -21932,10 +21932,10 @@
         <v>934</v>
       </c>
       <c r="AI182" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
     </row>
-    <row r="183" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>182</v>
       </c>
@@ -22036,7 +22036,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="184" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>183</v>
       </c>
@@ -22137,7 +22137,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="185" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>184</v>
       </c>
@@ -22238,7 +22238,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="186" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>185</v>
       </c>
@@ -22339,7 +22339,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="187" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>186</v>
       </c>
@@ -22440,7 +22440,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="188" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>187</v>
       </c>
@@ -22541,7 +22541,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="189" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>188</v>
       </c>
@@ -22621,7 +22621,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="190" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>189</v>
       </c>
@@ -22701,7 +22701,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="191" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>190</v>
       </c>
@@ -22778,7 +22778,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="192" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>191</v>
       </c>
@@ -22822,7 +22822,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="193" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>192</v>
       </c>
@@ -22867,7 +22867,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AI193" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>